<commit_message>
fix silent hardware result; fallback in qpu submmission(root cause, not symptom)
</commit_message>
<xml_diff>
--- a/MERGED_CSV/reports/SWARMGUARD_MODELING_LOG.xlsx
+++ b/MERGED_CSV/reports/SWARMGUARD_MODELING_LOG.xlsx
@@ -577,7 +577,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-09-24 08:39:29</t>
+          <t>2026-09-25 02:01:20</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -604,7 +604,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-09-24 08:40:43</t>
+          <t>2026-09-25 02:01:20</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -631,7 +631,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-09-24 08:43:23</t>
+          <t>2026-09-25 02:04:39</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -651,14 +651,14 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Trained 8 centralized model arms (~36 parameters each). QCNN achieved superior generalization vs controls.</t>
+          <t>Trained 4 arms x 2 branches (36 params each). Network: best test macro-F1 0.4382 by Proposed QCNN + Re-Upload / Capacity-Matched MLP / Matrix Product State (MPS); QCNN ranks 1 of 4 | Physical: best test macro-F1 0.4094 by Proposed QCNN + Re-Upload / Capacity-Matched MLP / Matrix Product State (MPS) / Hardware-Efficient VQC; QCNN ranks 1 of 4.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-09-24 08:49:46</t>
+          <t>2026-09-25 02:09:53</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -678,14 +678,14 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Benchmarked Rotosolve, SPSA, QNSPSA, ADAM. Rotosolve achieved rapid analytic convergence.</t>
+          <t>Benchmarked Rotosolve, SPSA, QNSPSA, ADAM (Param-Shift). Highest final accuracy 76.67% by QNSPSA (Network branch, X_test[:150]).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-09-24 08:52:22</t>
+          <t>2026-09-25 02:11:38</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -712,7 +712,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-24 08:52:35</t>
+          <t>2026-09-25 02:11:42</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -732,14 +732,14 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Implemented temporal alert fusion gate with Delta_t=3.0s; verified 4-outcome confusion matrix.</t>
+          <t>4-case fusion gate evaluated pointwise (Delta_t window not applied); 117/250 paired test samples (46.80%) assigned the correct fused state.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-09-24 08:53:22</t>
+          <t>2026-09-25 02:11:42</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>cross_check_ibm_quantum.py, swarmguard_modeling/qpu_executor.py</t>
+          <t>swarmguard_modeling/qpu_executor.py</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Submitted QCNN inference job to IBM Quantum hardware; confirmed hardware-simulated agreement within shot tolerance.</t>
+          <t>Real IBM job daqo4ueekp0c73ar2b7g on ibm_marrakesh: simulated &lt;Z&gt;=0.7207, hardware &lt;Z&gt;=0.5820 -&gt; COMPLETED (Outside Shot Tolerance).</t>
         </is>
       </c>
     </row>
@@ -795,6 +795,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -802,6 +803,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -945,6 +947,8 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -1212,6 +1216,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1219,6 +1224,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1578,6 +1584,8 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -1718,6 +1726,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1725,6 +1734,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1789,7 +1799,7 @@
         <v>36</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>76.86</v>
+        <v>76.56999999999999</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>78</v>
@@ -1798,11 +1808,11 @@
         <v>0.4382</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>3.64</v>
+        <v>46.34</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Hierarchical spatial locality (12-&gt;8-&gt;4-&gt;2-&gt;1); immune to barren plateaus; strong generalization</t>
+          <t>Train loss 0.5562 -&gt; 0.5531 over 60 SPSA iterations; predicts ATTACK for 100.0% of test (true rate 78.0%)</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1844,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Classical feedforward (12-&gt;2-&gt;2-&gt;1); constrained by 36-parameter linear bottleneck</t>
+          <t>Train loss 0.6932 -&gt; 0.5444 over 60 epochs; predicts ATTACK for 100.0% of test (true rate 78.0%)</t>
         </is>
       </c>
     </row>
@@ -1862,11 +1872,11 @@
         <v>0.4382</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>4.4</v>
+        <v>4.62</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Classical tensor network; captures 1D entanglement but lacks quantum superposition advantage</t>
+          <t>Train loss 0.7473 -&gt; 0.6446 over 15 epochs; predicts ATTACK for 100.0% of test (true rate 78.0%)</t>
         </is>
       </c>
     </row>
@@ -1885,20 +1895,20 @@
         <v>36</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>66.67</v>
+        <v>75.33</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.4</v>
+        <v>0.4297</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>1.57</v>
+        <v>40.94</v>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Non-hierarchical entangling ring; suffers from exponential gradient variance decay (Barren Plateau)</t>
+          <t>Train loss 0.6156 -&gt; 0.5806 over 60 SPSA iterations; predicts ATTACK for 97.3% of test (true rate 78.0%)</t>
         </is>
       </c>
     </row>
@@ -1926,11 +1936,11 @@
         <v>0.4094</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>3.61</v>
+        <v>45.92</v>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Hierarchical spatial locality (12-&gt;8-&gt;4-&gt;2-&gt;1); immune to barren plateaus; strong generalization</t>
+          <t>Train loss 0.7580 -&gt; 0.6987 over 60 SPSA iterations; predicts ATTACK for 100.0% of test (true rate 69.3%)</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1972,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Classical feedforward (12-&gt;2-&gt;2-&gt;1); constrained by 36-parameter linear bottleneck</t>
+          <t>Train loss 0.6931 -&gt; 0.6718 over 60 epochs; predicts ATTACK for 100.0% of test (true rate 69.3%)</t>
         </is>
       </c>
     </row>
@@ -1990,11 +2000,11 @@
         <v>0.4094</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>4.21</v>
+        <v>4.49</v>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Classical tensor network; captures 1D entanglement but lacks quantum superposition advantage</t>
+          <t>Train loss 0.7148 -&gt; 0.6842 over 15 epochs; predicts ATTACK for 100.0% of test (true rate 69.3%)</t>
         </is>
       </c>
     </row>
@@ -2022,11 +2032,11 @@
         <v>0.4094</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>1.5</v>
+        <v>41.6</v>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Non-hierarchical entangling ring; suffers from exponential gradient variance decay (Barren Plateau)</t>
+          <t>Train loss 0.8306 -&gt; 0.6697 over 60 SPSA iterations; predicts ATTACK for 100.0% of test (true rate 69.3%)</t>
         </is>
       </c>
     </row>
@@ -2066,6 +2076,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2073,6 +2084,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -2147,10 +2159,10 @@
         </is>
       </c>
       <c r="F7" s="11" t="n">
-        <v>79.33</v>
+        <v>75.33</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>179.81</v>
+        <v>147.03</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
@@ -2183,10 +2195,10 @@
         </is>
       </c>
       <c r="F8" s="12" t="n">
-        <v>76.67</v>
+        <v>76</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>16.01</v>
+        <v>18.1</v>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
@@ -2219,10 +2231,10 @@
         </is>
       </c>
       <c r="F9" s="11" t="n">
-        <v>78.67</v>
+        <v>76.67</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>12.09</v>
+        <v>13.3</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
@@ -2255,10 +2267,10 @@
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>76.67</v>
+        <v>76</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>157.86</v>
+        <v>130.91</v>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
@@ -2302,6 +2314,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2309,6 +2322,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -2378,17 +2392,17 @@
         <v>4</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>77.5</v>
+        <v>77</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>theta_bar_j = atan2( sum_k (n_k/N)*sin(theta_k,j), sum_k (n_k/N)*cos(theta_k,j) )</t>
+          <t>theta_bar_j = (P_j/2pi)*atan2( sum_k (n_k/N)*sin(2pi*theta_k,j/P_j), sum_k (n_k/N)*cos(2pi*theta_k,j/P_j) ), P_j = 2pi (Ry) / 4pi (CRz)</t>
         </is>
       </c>
     </row>
@@ -2412,17 +2426,17 @@
         <v>4</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>87.5</v>
+        <v>62</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>61.5</v>
+        <v>62</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>theta_bar_j = atan2( sum_k (n_k/N)*sin(theta_k,j), sum_k (n_k/N)*cos(theta_k,j) )</t>
+          <t>theta_bar_j = (P_j/2pi)*atan2( sum_k (n_k/N)*sin(2pi*theta_k,j/P_j), sum_k (n_k/N)*cos(2pi*theta_k,j/P_j) ), P_j = 2pi (Ry) / 4pi (CRz)</t>
         </is>
       </c>
     </row>
@@ -2461,6 +2475,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2468,6 +2483,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -2635,6 +2651,8 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -2686,10 +2704,10 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>0</v>
@@ -2701,7 +2719,7 @@
         <v>117</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>99.15000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -2736,13 +2754,13 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C17" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>0</v>
@@ -2751,7 +2769,7 @@
         <v>38</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>7.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
@@ -2761,13 +2779,13 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C18" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" s="12" t="n">
         <v>0</v>
@@ -2800,13 +2818,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2877,12 +2895,12 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>ibm_fez</t>
+          <t>ibm_marrakesh</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>ibm_hw_transpiled_1790220201</t>
+          <t>daqo4ueekp0c73ar2b7g</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -2892,27 +2910,27 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Depth 75</t>
+          <t>Depth 94</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>1024</t>
+          <t>1,024</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>0.6875</t>
+          <t>0.7207</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>0.6895</t>
+          <t>0.5820</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PASSED (Within Shot Tolerance)</t>
+          <t>COMPLETED (Outside Shot Tolerance)</t>
         </is>
       </c>
     </row>

</xml_diff>